<commit_message>
Deployed e81cfc6 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/downloads/en/periodicite-revues.xlsx
+++ b/downloads/en/periodicite-revues.xlsx
@@ -453,105 +453,105 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>One issue every two years</t>
+          <t>More than 4 issues/year</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Annual (1 issue/year)</t>
+          <t>Quarterly (4 issues/year)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C3" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Semiannual (2 issues/year)</t>
+          <t>Three issues per year</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>66</v>
+        <v>14</v>
       </c>
       <c r="C4" t="n">
-        <v>34</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Three issues per year</t>
+          <t>Semiannual (2 issues/year)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14</v>
+        <v>66</v>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Quarterly (4 issues/year)</t>
+          <t>Annual (1 issue/year)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C6" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>More than 4 issues/year</t>
+          <t>One issue every two years</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Irregular publication</t>
+          <t>Continuous publication</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Continuous publication</t>
+          <t>Irregular publication</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed 8a4bd96 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/downloads/en/periodicite-revues.xlsx
+++ b/downloads/en/periodicite-revues.xlsx
@@ -496,10 +496,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C5" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6">
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C6" t="n">
         <v>19</v>

</xml_diff>